<commit_message>
bug fix: ESPP has to use FMV for split-detection
</commit_message>
<xml_diff>
--- a/example/awv_report_2023.xlsx
+++ b/example/awv_report_2023.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>Meldezeitraum</t>
   </si>
@@ -53,9 +53,6 @@
     <t>US</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
     <t>Stückzahl</t>
   </si>
   <si>
@@ -72,9 +69,6 @@
   </si>
   <si>
     <t>US67066G1040</t>
-  </si>
-  <si>
-    <t>19</t>
   </si>
   <si>
     <t>USD</t>
@@ -440,7 +434,7 @@
   <cols>
     <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -493,8 +487,8 @@
       <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" t="s">
-        <v>12</v>
+      <c r="G2">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -532,13 +526,13 @@
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
@@ -553,7 +547,7 @@
         <v>7</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -567,10 +561,10 @@
         <v>41</v>
       </c>
       <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
         <v>17</v>
-      </c>
-      <c r="E2" t="s">
-        <v>18</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -578,11 +572,11 @@
       <c r="G2" t="s">
         <v>11</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2">
         <v>19</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>